<commit_message>
Update GOOD DAYS plan: Trio Fitness Hub, opening hours, variable menu
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q36W2VHzwtJBG7CP23uhQT
</commit_message>
<xml_diff>
--- a/gooddays/campaign/calendar.xlsx
+++ b/gooddays/campaign/calendar.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>في مكان بيهدّيك، وفي قهوة تستاهله. جود دايز جوّه [اسم المنتجع].</t>
+          <t>في مكان بيهدّيك، وفي قهوة تستاهله. جود دايز جوّه Trio Fitness Hub.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>بعد الـspa والتمرين</t>
+          <t>بعد التمرين</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1120,12 +1120,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>بعد الـspa: إيه اللي بتشتهيه؟</t>
+          <t>بعد التمرين: إيه اللي بتشتهيه؟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>جلسة مساج وبعدها قهوة؟ اتفقنا.</t>
+          <t>تمرين وبعده قهوة؟ اتفقنا.</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>بعد الـspa والتمرين</t>
+          <t>بعد التمرين</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>بعد الـspa والتمرين</t>
+          <t>بعد التمرين</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>الأكل الخفيف</t>
+          <t>منيو كبير ومتغيّر</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>أكل خفيف يشبعك [تأكيد المنيو]</t>
+          <t>منيو كبير ومتغيّر</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1627,11 +1627,7 @@
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
-        </is>
-      </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1649,7 +1645,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>الأكل الخفيف</t>
+          <t>منيو كبير ومتغيّر</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1674,7 +1670,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>كارت المنيو الخفيف (٣ أصناف)</t>
+          <t>منيو الأسبوع: ٣ مشروبات (ويتغيّر)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1711,7 +1707,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>الأكل الخفيف</t>
+          <t>منيو كبير ومتغيّر</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1769,7 +1765,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة: من ١٠ الصبح</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1794,7 +1790,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة في يومك: بنفتح ١٠ الصبح</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -1809,7 +1805,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>زورنا الصبح</t>
+          <t>زورنا من ١٠ الصبح</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
@@ -1831,7 +1827,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة: من ١٠ الصبح</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1856,7 +1852,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>صورة: كوباية الصبح مع الشمس</t>
+          <t>صورة: أول كوباية مع شمس الصبح (١٠ ص)</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1893,7 +1889,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة: من ١٠ الصبح</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1918,7 +1914,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>ريل: خطوات الصبح عندنا (٣ لقطات)</t>
+          <t>ريل: أول ساعة بعد الفتح (٣ لقطات)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1955,7 +1951,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة: من ١٠ الصبح</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1980,7 +1976,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>مين أول قهوة في يومه هنا؟</t>
+          <t>مين أول زبون عندنا الصبح؟</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
@@ -2013,7 +2009,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>طقوس الصباح</t>
+          <t>أول قهوة: من ١٠ الصبح</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2038,7 +2034,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>كارت: روتين ٣ خطوات للصبح</t>
+          <t>كارت: مواعيدنا: ١٠ صباحاً لـ١٢ منتصف الليل</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -2071,7 +2067,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>استراحة نص اليوم</t>
+          <t>سهرة لحد ١٢</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2096,12 +2092,12 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>الاستراحة نص اليوم</t>
+          <t>بنسهر معاك لحد ١٢</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>مش لازم تستنى الليل علشان ترتاح.</t>
+          <t>مش لازم تروّح بدري. القهوة مستنياك.</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2111,7 +2107,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>زورنا الضهر</t>
+          <t>زورنا بالليل</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
@@ -2133,7 +2129,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>استراحة نص اليوم</t>
+          <t>سهرة لحد ١٢</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2158,7 +2154,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>صورة: ترابيزة الضهر</t>
+          <t>صورة: الكافيه بالليل (إضاءة دافية)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
@@ -2191,7 +2187,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>استراحة نص اليوم</t>
+          <t>سهرة لحد ١٢</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2216,7 +2212,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>أنت بتاخد استراحة نص اليوم؟</t>
+          <t>أنت من ناس الصبح ولا الليل؟</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -2249,7 +2245,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>يوم ضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2274,12 +2270,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>يوم كامل لضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>قبل الـspa، بعد التمرين، قبل النوم.</t>
+          <t>قبل التمرين، بعده، وبالليل.</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2311,7 +2307,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>يوم ضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -2336,7 +2332,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>خريطة يوم الضيف (ساعات الزيارة) [تأكيد]</t>
+          <t>خريطة يوم كامل: تمرين ← قهوة ← سهرة</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -2351,11 +2347,7 @@
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
-        </is>
-      </c>
+      <c r="N31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2373,7 +2365,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>يوم ضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2398,7 +2390,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>ريل: يوم ضيف المنتجع (٨ لقطات)</t>
+          <t>ريل: يوم كامل في Trio Fitness Hub (٨ لقطات)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2435,7 +2427,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>يوم ضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -2460,7 +2452,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>مين ضيف المنتجع هنا؟</t>
+          <t>مين بيتمرن هنا ويعدّي علينا؟</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
@@ -2493,7 +2485,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>يوم ضيف المنتجع</t>
+          <t>يوم كامل في Trio Fitness Hub</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2518,7 +2510,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>كارت: ٣ أماكن تقعد فيها جوّه المنتجع</t>
+          <t>كارت: ٣ أماكن تقعد فيها عندنا</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2551,7 +2543,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>طاقة من غير تقل</t>
+          <t>الصحي جنب المعتاد</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2576,7 +2568,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>طاقة من غير تقل [تأكيد المنيو]</t>
+          <t>مشروبات صحية جنب القهوة المعتادة</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -2595,11 +2587,7 @@
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr">
-        <is>
-          <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
-        </is>
-      </c>
+      <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2617,7 +2605,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>طاقة من غير تقل</t>
+          <t>الصحي جنب المعتاد</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2642,7 +2630,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>كارت: مشروب الطاقة (المكونات فقط)</t>
+          <t>كارت: مشروب صحي من منيو الأسبوع (المكونات فقط)</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -2675,7 +2663,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>طاقة من غير تقل</t>
+          <t>الصحي جنب المعتاد</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2733,7 +2721,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>طاقة من غير تقل</t>
+          <t>الصحي جنب المعتاد</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
GOOD DAYS plan: Facebook + Instagram only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q36W2VHzwtJBG7CP23uhQT
</commit_message>
<xml_diff>
--- a/gooddays/campaign/calendar.xlsx
+++ b/gooddays/campaign/calendar.xlsx
@@ -548,12 +548,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -986,12 +986,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1292,12 +1292,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1478,12 +1478,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1598,12 +1598,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1722,12 +1722,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1780,12 +1780,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1966,12 +1966,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -2082,12 +2082,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -2202,12 +2202,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2260,12 +2260,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -2442,12 +2442,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2558,12 +2558,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2736,12 +2736,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2794,12 +2794,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2914,12 +2914,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -3030,12 +3030,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -3212,12 +3212,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -3270,12 +3270,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>ريلز إنستجرام + فيسبوك + تيك توك</t>
+          <t>ريلز إنستجرام + ريلز فيسبوك</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -3452,12 +3452,12 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>تويتة</t>
+          <t>بوست نصي/تفاعلي</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>فيسبوك + ستوري إنستجرام</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">

</xml_diff>

<commit_message>
GOOD DAYS: 18 static posts (AR+EN), copy for 24 text posts, captions, reel briefs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q36W2VHzwtJBG7CP23uhQT
</commit_message>
<xml_diff>
--- a/gooddays/campaign/calendar.xlsx
+++ b/gooddays/campaign/calendar.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -442,7 +442,8 @@
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,6 +514,11 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Files / copy</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Before publishing</t>
         </is>
       </c>
@@ -577,7 +583,12 @@
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -639,7 +650,12 @@
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w01_mon_reset.png</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -705,7 +721,12 @@
           <t>جاهز</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk01_tue_gym_to_cafe</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -767,7 +788,12 @@
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -829,7 +855,12 @@
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -891,7 +922,12 @@
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
-      <c r="N7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w02_mon_quiet_corner.png</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -953,7 +989,12 @@
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk02_tue_listen</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1015,7 +1056,12 @@
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1077,7 +1123,12 @@
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w02_thu_hour_here.png</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1139,7 +1190,12 @@
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr"/>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1201,7 +1257,12 @@
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w03_mon_earned_it.png</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1259,7 +1320,12 @@
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr"/>
-      <c r="N13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1321,7 +1387,12 @@
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
-      <c r="N14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1383,7 +1454,12 @@
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w04_mon_sun.png</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1445,7 +1521,12 @@
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk04_tue_sun</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1503,7 +1584,12 @@
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
-      <c r="N17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1563,6 +1649,11 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
+          <t>posts/out/ar|en/w04_thu_outside.png</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
           <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
         </is>
       </c>
@@ -1627,7 +1718,12 @@
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1689,7 +1785,12 @@
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
-      <c r="N20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w05_mon_menu.png</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1747,7 +1848,12 @@
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1809,7 +1915,12 @@
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1871,7 +1982,12 @@
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr"/>
-      <c r="N23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w06_mon_first_coffee.png</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1933,7 +2049,12 @@
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk06_tue_first_hour</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1991,7 +2112,12 @@
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2034,7 +2160,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>كارت: مواعيدنا: ١٠ صباحاً لـ١٢ منتصف الليل</t>
+          <t>مواعيدنا: ١٠ صباحاً لـ١٢ منتصف الليل</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
@@ -2049,7 +2175,12 @@
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w06_thu_hours.png</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2111,7 +2242,12 @@
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2169,7 +2305,12 @@
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w07_mon_late.png</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2227,7 +2368,12 @@
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2289,7 +2435,12 @@
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2347,7 +2498,12 @@
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w08_mon_whole_day.png</t>
+        </is>
+      </c>
+      <c r="O31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2409,7 +2565,12 @@
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr"/>
-      <c r="N32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk08_tue_full_day</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2467,7 +2628,12 @@
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2510,7 +2676,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>كارت: ٣ أماكن تقعد فيها عندنا</t>
+          <t>مش لازم تكون عضو</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
@@ -2525,7 +2691,12 @@
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w08_thu_no_membership.png</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2587,7 +2758,12 @@
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2630,7 +2806,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>كارت: مشروب صحي من منيو الأسبوع (المكونات فقط)</t>
+          <t>الصحي جنب المعتاد</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
@@ -2645,7 +2821,12 @@
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w09_mon_healthy.png</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2703,7 +2884,12 @@
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk09_tue_pour</t>
+        </is>
+      </c>
+      <c r="O37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2761,7 +2947,12 @@
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2823,7 +3014,12 @@
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2881,7 +3077,12 @@
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w10_mon_company.png</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2939,7 +3140,12 @@
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2982,7 +3188,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>كارت: ٣ أفكار لقعدة جماعية</t>
+          <t>جيب صحابك</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
@@ -2997,7 +3203,12 @@
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w10_thu_bring.png</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3059,7 +3270,12 @@
         </is>
       </c>
       <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3102,7 +3318,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>كارت: كارت الولاء (فكرة) [تأكيد]</t>
+          <t>كل زيارة بتبقى عادة</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
@@ -3119,9 +3335,10 @@
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
-        </is>
-      </c>
+          <t>posts/out/ar|en/w11_mon_habit.png</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3179,7 +3396,12 @@
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr"/>
-      <c r="N45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk11_tue_repeat</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3237,7 +3459,12 @@
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr"/>
-      <c r="N46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3299,7 +3526,12 @@
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr"/>
-      <c r="N47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3361,7 +3593,12 @@
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr"/>
-      <c r="N48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w12_mon_earned_part.png</t>
+        </is>
+      </c>
+      <c r="O48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3419,7 +3656,12 @@
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr"/>
-      <c r="N49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>reels: wk12_tue_best_of</t>
+        </is>
+      </c>
+      <c r="O49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3462,7 +3704,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>شكراً + عرض الختام [تأكيد]</t>
+          <t>شكراً + مواعيد الشغل</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
@@ -3479,9 +3721,10 @@
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>تأكيد المنيو/العرض/الساعات قبل النشر</t>
-        </is>
-      </c>
+          <t>content.md (text posts)</t>
+        </is>
+      </c>
+      <c r="O50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3539,7 +3782,12 @@
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr"/>
-      <c r="N51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>posts/out/ar|en/w12_thu_thanks.png</t>
+        </is>
+      </c>
+      <c r="O51" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>